<commit_message>
first phase server updated
</commit_message>
<xml_diff>
--- a/hostel_management_Frontend/public/sample1.xlsx
+++ b/hostel_management_Frontend/public/sample1.xlsx
@@ -32,46 +32,46 @@
     <t>s.no</t>
   </si>
   <si>
-    <t>Member ID</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>Degree</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Expiry Date</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Hostel Name</t>
-  </si>
-  <si>
-    <t>Room No</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Parant/Guardian Name</t>
-  </si>
-  <si>
-    <t>Parant/Guardian Contact</t>
-  </si>
-  <si>
-    <t>Remark</t>
+    <t xml:space="preserve">memberid </t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>degree</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>expirydate</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>hostel_id</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>parentname</t>
+  </si>
+  <si>
+    <t>parentcontact</t>
+  </si>
+  <si>
+    <t>remarks</t>
   </si>
   <si>
     <t>2cqr automation</t>
@@ -743,7 +743,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1077,7 +1077,7 @@
     <col min="17" max="17" width="12.9074074074074" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" ht="28.8" spans="1:15">
+    <row r="1" customFormat="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
student registration pagination added and parentemail added
</commit_message>
<xml_diff>
--- a/hostel_management_Frontend/public/sample1.xlsx
+++ b/hostel_management_Frontend/public/sample1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>s.no</t>
   </si>
@@ -68,6 +68,9 @@
     <t>parentname</t>
   </si>
   <si>
+    <t>parentemail</t>
+  </si>
+  <si>
     <t>parentcontact</t>
   </si>
   <si>
@@ -96,6 +99,9 @@
   </si>
   <si>
     <t>arun</t>
+  </si>
+  <si>
+    <t>muthiah1006@gmail.com</t>
   </si>
   <si>
     <t>Remarks</t>
@@ -737,7 +743,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -748,6 +754,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1067,17 +1075,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="2" max="9" width="17.6296296296296" customWidth="1"/>
-    <col min="10" max="14" width="15.1759259259259" customWidth="1"/>
-    <col min="15" max="15" width="12.9074074074074" customWidth="1"/>
-    <col min="16" max="16" width="15.1759259259259" customWidth="1"/>
-    <col min="17" max="17" width="12.9074074074074" customWidth="1"/>
+    <col min="10" max="15" width="15.1759259259259" customWidth="1"/>
+    <col min="16" max="16" width="12.9074074074074" customWidth="1"/>
+    <col min="17" max="17" width="15.1759259259259" customWidth="1"/>
+    <col min="18" max="18" width="12.9074074074074" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:15">
+    <row r="1" customFormat="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1117,14 +1125,17 @@
       <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" customFormat="1" spans="1:15">
+    <row r="2" customFormat="1" spans="1:16">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1132,46 +1143,49 @@
         <v>567</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2">
         <v>9791344113</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" s="4">
         <v>46016</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2">
         <v>100</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2">
+        <v>23</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2">
         <v>9791344113</v>
       </c>
-      <c r="O2" t="s">
-        <v>23</v>
+      <c r="P2" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:15">
+    <row r="3" customFormat="1" spans="1:16">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1179,49 +1193,54 @@
         <v>789</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F3">
         <v>9791344112</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" s="4">
         <v>46016</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K3">
         <v>100</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3">
+        <v>23</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3">
         <v>9791344113</v>
       </c>
-      <c r="O3" t="s">
-        <v>23</v>
+      <c r="P3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" display="2cqr1@gmail.com"/>
     <hyperlink ref="G3" r:id="rId1" display="2cqr1@gmail.com"/>
+    <hyperlink ref="N2" r:id="rId2" display="muthiah1006@gmail.com" tooltip="mailto:muthiah1006@gmail.com"/>
+    <hyperlink ref="N3" r:id="rId2" display="muthiah1006@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>